<commit_message>
Refine the dance spreadsheet's hour-summary tabs: staleness footer, caller grouping, number formatting
Adds a "Calculated at" timestamp plus a live NOW()-based "Status" formula
that flags each tab as possibly stale once the workbook is recalculated,
since these tabs are static snapshots that go stale if a day sheet is
edited without re-running the generator. Also groups "By Caller" columns
into headline callers (sorted by descending hours) and GCA-showcase-only
callers, with a divider border between the two groups, and rounds hour
values before writing them so a whole number renders as "1" instead of a
near-integer float displaying as "1."

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content/backtrack2abq/data/dance-schedule.xlsx
+++ b/content/backtrack2abq/data/dance-schedule.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="283" uniqueCount="238">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="287" uniqueCount="240">
   <si>
     <t>Time</t>
   </si>
@@ -732,109 +732,115 @@
     <t>Generated by scripts/generate-dance-schedule-hour-tabs.ts — re-run after editing any day's schedule.</t>
   </si>
   <si>
+    <t>Calculated at:</t>
+  </si>
+  <si>
+    <t>Status:</t>
+  </si>
+  <si>
+    <t>Kris Jensen</t>
+  </si>
+  <si>
+    <t>Sandie Bryant</t>
+  </si>
+  <si>
+    <t>Ted Lizotte</t>
+  </si>
+  <si>
+    <t>Michael Kellogg</t>
+  </si>
+  <si>
+    <t>Vic Ceder</t>
+  </si>
+  <si>
+    <t>Justin Russell</t>
+  </si>
+  <si>
+    <t>Rob French</t>
+  </si>
+  <si>
+    <t>Don Moger</t>
+  </si>
+  <si>
+    <t>Barry Clasper</t>
+  </si>
+  <si>
+    <t>Dayle Hodge</t>
+  </si>
+  <si>
+    <t>Dave Hutchinson</t>
+  </si>
+  <si>
+    <t>Wendy VanderMeulen</t>
+  </si>
+  <si>
+    <t>Brian Crawford</t>
+  </si>
+  <si>
+    <t>Allan Hurst</t>
+  </si>
+  <si>
+    <t>Kurt Gollhardt</t>
+  </si>
+  <si>
+    <t>Rick Hawes</t>
+  </si>
+  <si>
+    <t>Ett McAtee</t>
+  </si>
+  <si>
+    <t>Karla Westphal</t>
+  </si>
+  <si>
     <t>All Callers</t>
   </si>
   <si>
-    <t>Allan Hurst</t>
-  </si>
-  <si>
-    <t>Barry Clasper</t>
+    <t>Jenn Engimann</t>
+  </si>
+  <si>
+    <t>Marge Coahran</t>
+  </si>
+  <si>
+    <t>Terri Sherrer</t>
   </si>
   <si>
     <t>Bill van Melle</t>
   </si>
   <si>
-    <t>Brian Crawford</t>
-  </si>
-  <si>
     <t>Brian Jarvis</t>
   </si>
   <si>
-    <t>Dave Hutchinson</t>
-  </si>
-  <si>
     <t>David Hartman</t>
   </si>
   <si>
-    <t>Dayle Hodge</t>
-  </si>
-  <si>
-    <t>Don Moger</t>
-  </si>
-  <si>
-    <t>Ett McAtee</t>
+    <t>Jane Clewe</t>
+  </si>
+  <si>
+    <t>Janienne Alexander</t>
+  </si>
+  <si>
+    <t>John Hawley</t>
+  </si>
+  <si>
+    <t>Michael Levy</t>
+  </si>
+  <si>
+    <t>Michael Maltenfort</t>
+  </si>
+  <si>
+    <t>Patrick Aubert</t>
+  </si>
+  <si>
+    <t>Ryo Sasaki</t>
+  </si>
+  <si>
+    <t>Tim Stephens</t>
   </si>
   <si>
     <t>Greg Moore</t>
   </si>
   <si>
-    <t>Jane Clewe</t>
-  </si>
-  <si>
-    <t>Janienne Alexander</t>
-  </si>
-  <si>
-    <t>Jenn Engimann</t>
-  </si>
-  <si>
-    <t>John Hawley</t>
-  </si>
-  <si>
-    <t>Justin Russell</t>
-  </si>
-  <si>
     <t>Karin Rabe</t>
-  </si>
-  <si>
-    <t>Karla Westphal</t>
-  </si>
-  <si>
-    <t>Kris Jensen</t>
-  </si>
-  <si>
-    <t>Kurt Gollhardt</t>
-  </si>
-  <si>
-    <t>Marge Coahran</t>
-  </si>
-  <si>
-    <t>Michael Kellogg</t>
-  </si>
-  <si>
-    <t>Michael Levy</t>
-  </si>
-  <si>
-    <t>Michael Maltenfort</t>
-  </si>
-  <si>
-    <t>Patrick Aubert</t>
-  </si>
-  <si>
-    <t>Rick Hawes</t>
-  </si>
-  <si>
-    <t>Rob French</t>
-  </si>
-  <si>
-    <t>Ryo Sasaki</t>
-  </si>
-  <si>
-    <t>Sandie Bryant</t>
-  </si>
-  <si>
-    <t>Ted Lizotte</t>
-  </si>
-  <si>
-    <t>Terri Sherrer</t>
-  </si>
-  <si>
-    <t>Tim Stephens</t>
-  </si>
-  <si>
-    <t>Vic Ceder</t>
-  </si>
-  <si>
-    <t>Wendy VanderMeulen</t>
   </si>
 </sst>
 </file>
@@ -895,7 +901,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -918,11 +924,18 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="medium"/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -946,6 +959,8 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2122,7 +2137,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:M9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="2" max="2" width="9" style="8" customWidth="1"/>
@@ -2361,6 +2376,45 @@
       <c r="L7" s="8"/>
       <c r="M7" s="8"/>
     </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>203</v>
+      </c>
+      <c r="B8" s="8">
+        <v>46240.62467592592</v>
+      </c>
+      <c r="C8" s="8"/>
+      <c r="D8" s="8"/>
+      <c r="E8" s="8"/>
+      <c r="F8" s="8"/>
+      <c r="G8" s="8"/>
+      <c r="H8" s="8"/>
+      <c r="I8" s="8"/>
+      <c r="J8" s="8"/>
+      <c r="K8" s="8"/>
+      <c r="L8" s="8"/>
+      <c r="M8" s="8"/>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>204</v>
+      </c>
+      <c r="B9" s="8" t="str">
+        <f>IF(NOW()&gt;B8+TIME(0,2,0),"⚠ Recalculated since Calculated-at — totals may be stale, re-run the generator script","✓ Up to date as of the Calculated-at time above")</f>
+        <v>✓ Up to date as of the Calculated-at time above</v>
+      </c>
+      <c r="C9" s="8"/>
+      <c r="D9" s="8"/>
+      <c r="E9" s="8"/>
+      <c r="F9" s="8"/>
+      <c r="G9" s="8"/>
+      <c r="H9" s="8"/>
+      <c r="I9" s="8"/>
+      <c r="J9" s="8"/>
+      <c r="K9" s="8"/>
+      <c r="L9" s="8"/>
+      <c r="M9" s="8"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -2369,7 +2423,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AL7"/>
+  <dimension ref="A1:AL9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="2" max="2" width="9" style="8" customWidth="1"/>
@@ -2416,112 +2470,112 @@
         <v>186</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="G1" s="10" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="H1" s="10" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="I1" s="10" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="J1" s="10" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="K1" s="10" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="L1" s="10" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="M1" s="10" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="N1" s="10" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="O1" s="10" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="P1" s="10" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="Q1" s="10" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="R1" s="10" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="S1" s="10" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="T1" s="10" t="s">
-        <v>221</v>
+        <v>197</v>
       </c>
       <c r="U1" s="10" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="V1" s="10" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="W1" s="10" t="s">
-        <v>224</v>
-      </c>
-      <c r="X1" s="10" t="s">
         <v>225</v>
       </c>
+      <c r="X1" s="11" t="s">
+        <v>226</v>
+      </c>
       <c r="Y1" s="10" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="Z1" s="10" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="AA1" s="10" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="AB1" s="10" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="AC1" s="10" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="AD1" s="10" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="AE1" s="10" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AF1" s="10" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="AG1" s="10" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="AH1" s="10" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="AI1" s="10" t="s">
-        <v>197</v>
+        <v>237</v>
       </c>
       <c r="AJ1" s="10" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="AK1" s="10" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="AL1" s="10" t="s">
         <v>198</v>
@@ -2532,40 +2586,40 @@
         <v>199</v>
       </c>
       <c r="B2" s="8">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="C2" s="8">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D2" s="8">
+        <v>5</v>
+      </c>
+      <c r="E2" s="8">
+        <v>4.5</v>
+      </c>
+      <c r="F2" s="8">
+        <v>4</v>
+      </c>
+      <c r="G2" s="8">
+        <v>5</v>
+      </c>
+      <c r="H2" s="8">
+        <v>5</v>
+      </c>
+      <c r="I2" s="8">
+        <v>5</v>
+      </c>
+      <c r="J2" s="8">
         <v>3</v>
       </c>
-      <c r="E2" s="8">
-        <v>0</v>
-      </c>
-      <c r="F2" s="8">
-        <v>0</v>
-      </c>
-      <c r="G2" s="8">
-        <v>0</v>
-      </c>
-      <c r="H2" s="8">
-        <v>1</v>
-      </c>
-      <c r="I2" s="8">
-        <v>0</v>
-      </c>
-      <c r="J2" s="8">
-        <v>0</v>
-      </c>
       <c r="K2" s="8">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L2" s="8">
         <v>1</v>
       </c>
       <c r="M2" s="8">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="N2" s="8">
         <v>0</v>
@@ -2580,16 +2634,16 @@
         <v>0</v>
       </c>
       <c r="R2" s="8">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="S2" s="8">
         <v>0</v>
       </c>
       <c r="T2" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U2" s="8">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="V2" s="8">
         <v>0</v>
@@ -2597,8 +2651,8 @@
       <c r="W2" s="8">
         <v>0</v>
       </c>
-      <c r="X2" s="8">
-        <v>4.5</v>
+      <c r="X2" s="12">
+        <v>0.5</v>
       </c>
       <c r="Y2" s="8">
         <v>0</v>
@@ -2613,31 +2667,31 @@
         <v>0</v>
       </c>
       <c r="AC2" s="8">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AD2" s="8">
         <v>0</v>
       </c>
       <c r="AE2" s="8">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="AF2" s="8">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AG2" s="8">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="AH2" s="8">
         <v>0</v>
       </c>
       <c r="AI2" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AJ2" s="8">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="AK2" s="8">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AL2" s="8">
         <v>47</v>
@@ -2648,73 +2702,73 @@
         <v>200</v>
       </c>
       <c r="B3" s="8">
+        <v>4</v>
+      </c>
+      <c r="C3" s="8">
+        <v>6</v>
+      </c>
+      <c r="D3" s="8">
+        <v>5</v>
+      </c>
+      <c r="E3" s="8">
+        <v>6</v>
+      </c>
+      <c r="F3" s="8">
+        <v>4</v>
+      </c>
+      <c r="G3" s="8">
+        <v>4</v>
+      </c>
+      <c r="H3" s="8">
+        <v>4</v>
+      </c>
+      <c r="I3" s="8">
+        <v>4</v>
+      </c>
+      <c r="J3" s="8">
+        <v>3</v>
+      </c>
+      <c r="K3" s="8">
+        <v>1.5</v>
+      </c>
+      <c r="L3" s="8">
+        <v>1</v>
+      </c>
+      <c r="M3" s="8">
+        <v>0</v>
+      </c>
+      <c r="N3" s="8">
+        <v>0</v>
+      </c>
+      <c r="O3" s="8">
+        <v>0</v>
+      </c>
+      <c r="P3" s="8">
+        <v>1</v>
+      </c>
+      <c r="Q3" s="8">
+        <v>1</v>
+      </c>
+      <c r="R3" s="8">
+        <v>0</v>
+      </c>
+      <c r="S3" s="8">
+        <v>0.5</v>
+      </c>
+      <c r="T3" s="8">
+        <v>0</v>
+      </c>
+      <c r="U3" s="8">
         <v>0.75</v>
       </c>
-      <c r="C3" s="8">
-        <v>0</v>
-      </c>
-      <c r="D3" s="8">
-        <v>3</v>
-      </c>
-      <c r="E3" s="8">
-        <v>0</v>
-      </c>
-      <c r="F3" s="8">
-        <v>0</v>
-      </c>
-      <c r="G3" s="8">
-        <v>0</v>
-      </c>
-      <c r="H3" s="8">
-        <v>1</v>
-      </c>
-      <c r="I3" s="8">
-        <v>0</v>
-      </c>
-      <c r="J3" s="8">
-        <v>1.5</v>
-      </c>
-      <c r="K3" s="8">
-        <v>4</v>
-      </c>
-      <c r="L3" s="8">
-        <v>0</v>
-      </c>
-      <c r="M3" s="8">
-        <v>0</v>
-      </c>
-      <c r="N3" s="8">
-        <v>0</v>
-      </c>
-      <c r="O3" s="8">
-        <v>0</v>
-      </c>
-      <c r="P3" s="8">
+      <c r="V3" s="8">
         <v>0.5</v>
-      </c>
-      <c r="Q3" s="8">
-        <v>0</v>
-      </c>
-      <c r="R3" s="8">
-        <v>4</v>
-      </c>
-      <c r="S3" s="8">
-        <v>0</v>
-      </c>
-      <c r="T3" s="8">
-        <v>0.5</v>
-      </c>
-      <c r="U3" s="8">
-        <v>4</v>
-      </c>
-      <c r="V3" s="8">
-        <v>1</v>
       </c>
       <c r="W3" s="8">
         <v>0.5</v>
       </c>
-      <c r="X3" s="8">
-        <v>6</v>
+      <c r="X3" s="12">
+        <v>0</v>
       </c>
       <c r="Y3" s="8">
         <v>0</v>
@@ -2726,19 +2780,19 @@
         <v>0</v>
       </c>
       <c r="AB3" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AC3" s="8">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="AD3" s="8">
         <v>0</v>
       </c>
       <c r="AE3" s="8">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AF3" s="8">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AG3" s="8">
         <v>0</v>
@@ -2750,7 +2804,7 @@
         <v>0</v>
       </c>
       <c r="AJ3" s="8">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="AK3" s="8">
         <v>0</v>
@@ -2764,73 +2818,73 @@
         <v>201</v>
       </c>
       <c r="B4" s="8">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="C4" s="8">
-        <v>1.5</v>
+        <v>4</v>
       </c>
       <c r="D4" s="8">
+        <v>4</v>
+      </c>
+      <c r="E4" s="8">
         <v>3</v>
       </c>
-      <c r="E4" s="8">
-        <v>0.5</v>
-      </c>
       <c r="F4" s="8">
+        <v>4.5</v>
+      </c>
+      <c r="G4" s="8">
+        <v>3</v>
+      </c>
+      <c r="H4" s="8">
+        <v>3</v>
+      </c>
+      <c r="I4" s="8">
         <v>2</v>
-      </c>
-      <c r="G4" s="8">
-        <v>0.5</v>
-      </c>
-      <c r="H4" s="8">
-        <v>1</v>
-      </c>
-      <c r="I4" s="8">
-        <v>0.5</v>
       </c>
       <c r="J4" s="8">
         <v>3</v>
       </c>
       <c r="K4" s="8">
+        <v>3</v>
+      </c>
+      <c r="L4" s="8">
+        <v>1</v>
+      </c>
+      <c r="M4" s="8">
+        <v>0</v>
+      </c>
+      <c r="N4" s="8">
         <v>2</v>
       </c>
-      <c r="L4" s="8">
-        <v>0</v>
-      </c>
-      <c r="M4" s="8">
-        <v>0.25</v>
-      </c>
-      <c r="N4" s="8">
+      <c r="O4" s="8">
+        <v>1.5</v>
+      </c>
+      <c r="P4" s="8">
         <v>0.5</v>
-      </c>
-      <c r="O4" s="8">
-        <v>0.5</v>
-      </c>
-      <c r="P4" s="8">
-        <v>0</v>
       </c>
       <c r="Q4" s="8">
         <v>0.5</v>
       </c>
       <c r="R4" s="8">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="S4" s="8">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="T4" s="8">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="U4" s="8">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="V4" s="8">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="W4" s="8">
         <v>0</v>
       </c>
-      <c r="X4" s="8">
-        <v>3</v>
+      <c r="X4" s="12">
+        <v>0</v>
       </c>
       <c r="Y4" s="8">
         <v>0.5</v>
@@ -2845,31 +2899,31 @@
         <v>0.5</v>
       </c>
       <c r="AC4" s="8">
-        <v>3</v>
+        <v>0.5</v>
       </c>
       <c r="AD4" s="8">
         <v>0.5</v>
       </c>
       <c r="AE4" s="8">
-        <v>4</v>
+        <v>0.5</v>
       </c>
       <c r="AF4" s="8">
-        <v>4</v>
+        <v>0.5</v>
       </c>
       <c r="AG4" s="8">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="AH4" s="8">
         <v>0.5</v>
       </c>
       <c r="AI4" s="8">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="AJ4" s="8">
-        <v>4.5</v>
+        <v>0.25</v>
       </c>
       <c r="AK4" s="8">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="AL4" s="8">
         <v>46.5</v>
@@ -2880,73 +2934,73 @@
         <v>198</v>
       </c>
       <c r="B5" s="10">
-        <v>0.75</v>
+        <v>14</v>
       </c>
       <c r="C5" s="10">
+        <v>14</v>
+      </c>
+      <c r="D5" s="10">
+        <v>14</v>
+      </c>
+      <c r="E5" s="10">
+        <v>13.5</v>
+      </c>
+      <c r="F5" s="10">
+        <v>12.5</v>
+      </c>
+      <c r="G5" s="10">
+        <v>12</v>
+      </c>
+      <c r="H5" s="10">
+        <v>12</v>
+      </c>
+      <c r="I5" s="10">
+        <v>11</v>
+      </c>
+      <c r="J5" s="10">
+        <v>9</v>
+      </c>
+      <c r="K5" s="10">
+        <v>4.5</v>
+      </c>
+      <c r="L5" s="10">
+        <v>3</v>
+      </c>
+      <c r="M5" s="10">
+        <v>3</v>
+      </c>
+      <c r="N5" s="10">
+        <v>2</v>
+      </c>
+      <c r="O5" s="10">
         <v>1.5</v>
       </c>
-      <c r="D5" s="10">
-        <v>9</v>
-      </c>
-      <c r="E5" s="10">
-        <v>0.5</v>
-      </c>
-      <c r="F5" s="10">
-        <v>2</v>
-      </c>
-      <c r="G5" s="10">
-        <v>0.5</v>
-      </c>
-      <c r="H5" s="10">
-        <v>3</v>
-      </c>
-      <c r="I5" s="10">
-        <v>0.5</v>
-      </c>
-      <c r="J5" s="10">
-        <v>4.5</v>
-      </c>
-      <c r="K5" s="10">
-        <v>11</v>
-      </c>
-      <c r="L5" s="10">
+      <c r="P5" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="Q5" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="R5" s="10">
         <v>1</v>
       </c>
-      <c r="M5" s="10">
-        <v>0.25</v>
-      </c>
-      <c r="N5" s="10">
-        <v>0.5</v>
-      </c>
-      <c r="O5" s="10">
-        <v>0.5</v>
-      </c>
-      <c r="P5" s="10">
-        <v>0.5</v>
-      </c>
-      <c r="Q5" s="10">
-        <v>0.5</v>
-      </c>
-      <c r="R5" s="10">
-        <v>12</v>
-      </c>
       <c r="S5" s="10">
-        <v>0.25</v>
+        <v>1</v>
       </c>
       <c r="T5" s="10">
         <v>1</v>
       </c>
       <c r="U5" s="10">
-        <v>14</v>
+        <v>0.75</v>
       </c>
       <c r="V5" s="10">
-        <v>1.5</v>
+        <v>0.5</v>
       </c>
       <c r="W5" s="10">
         <v>0.5</v>
       </c>
-      <c r="X5" s="10">
-        <v>13.5</v>
+      <c r="X5" s="11">
+        <v>0.5</v>
       </c>
       <c r="Y5" s="10">
         <v>0.5</v>
@@ -2958,19 +3012,19 @@
         <v>0.5</v>
       </c>
       <c r="AB5" s="10">
-        <v>1.5</v>
+        <v>0.5</v>
       </c>
       <c r="AC5" s="10">
-        <v>12</v>
+        <v>0.5</v>
       </c>
       <c r="AD5" s="10">
         <v>0.5</v>
       </c>
       <c r="AE5" s="10">
-        <v>14</v>
+        <v>0.5</v>
       </c>
       <c r="AF5" s="10">
-        <v>14</v>
+        <v>0.5</v>
       </c>
       <c r="AG5" s="10">
         <v>0.5</v>
@@ -2979,13 +3033,13 @@
         <v>0.5</v>
       </c>
       <c r="AI5" s="10">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="AJ5" s="10">
-        <v>12.5</v>
+        <v>0.25</v>
       </c>
       <c r="AK5" s="10">
-        <v>3</v>
+        <v>0.25</v>
       </c>
       <c r="AL5" s="10">
         <v>140.25</v>
@@ -3033,6 +3087,95 @@
       <c r="AK7" s="8"/>
       <c r="AL7" s="8"/>
     </row>
+    <row r="8" spans="1:38" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>203</v>
+      </c>
+      <c r="B8" s="8">
+        <v>46240.62467592592</v>
+      </c>
+      <c r="C8" s="8"/>
+      <c r="D8" s="8"/>
+      <c r="E8" s="8"/>
+      <c r="F8" s="8"/>
+      <c r="G8" s="8"/>
+      <c r="H8" s="8"/>
+      <c r="I8" s="8"/>
+      <c r="J8" s="8"/>
+      <c r="K8" s="8"/>
+      <c r="L8" s="8"/>
+      <c r="M8" s="8"/>
+      <c r="N8" s="8"/>
+      <c r="O8" s="8"/>
+      <c r="P8" s="8"/>
+      <c r="Q8" s="8"/>
+      <c r="R8" s="8"/>
+      <c r="S8" s="8"/>
+      <c r="T8" s="8"/>
+      <c r="U8" s="8"/>
+      <c r="V8" s="8"/>
+      <c r="W8" s="8"/>
+      <c r="X8" s="8"/>
+      <c r="Y8" s="8"/>
+      <c r="Z8" s="8"/>
+      <c r="AA8" s="8"/>
+      <c r="AB8" s="8"/>
+      <c r="AC8" s="8"/>
+      <c r="AD8" s="8"/>
+      <c r="AE8" s="8"/>
+      <c r="AF8" s="8"/>
+      <c r="AG8" s="8"/>
+      <c r="AH8" s="8"/>
+      <c r="AI8" s="8"/>
+      <c r="AJ8" s="8"/>
+      <c r="AK8" s="8"/>
+      <c r="AL8" s="8"/>
+    </row>
+    <row r="9" spans="1:38" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>204</v>
+      </c>
+      <c r="B9" s="8" t="str">
+        <f>IF(NOW()&gt;B8+TIME(0,2,0),"⚠ Recalculated since Calculated-at — totals may be stale, re-run the generator script","✓ Up to date as of the Calculated-at time above")</f>
+        <v>✓ Up to date as of the Calculated-at time above</v>
+      </c>
+      <c r="C9" s="8"/>
+      <c r="D9" s="8"/>
+      <c r="E9" s="8"/>
+      <c r="F9" s="8"/>
+      <c r="G9" s="8"/>
+      <c r="H9" s="8"/>
+      <c r="I9" s="8"/>
+      <c r="J9" s="8"/>
+      <c r="K9" s="8"/>
+      <c r="L9" s="8"/>
+      <c r="M9" s="8"/>
+      <c r="N9" s="8"/>
+      <c r="O9" s="8"/>
+      <c r="P9" s="8"/>
+      <c r="Q9" s="8"/>
+      <c r="R9" s="8"/>
+      <c r="S9" s="8"/>
+      <c r="T9" s="8"/>
+      <c r="U9" s="8"/>
+      <c r="V9" s="8"/>
+      <c r="W9" s="8"/>
+      <c r="X9" s="8"/>
+      <c r="Y9" s="8"/>
+      <c r="Z9" s="8"/>
+      <c r="AA9" s="8"/>
+      <c r="AB9" s="8"/>
+      <c r="AC9" s="8"/>
+      <c r="AD9" s="8"/>
+      <c r="AE9" s="8"/>
+      <c r="AF9" s="8"/>
+      <c r="AG9" s="8"/>
+      <c r="AH9" s="8"/>
+      <c r="AI9" s="8"/>
+      <c r="AJ9" s="8"/>
+      <c r="AK9" s="8"/>
+      <c r="AL9" s="8"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>